<commit_message>
Add regression calculation sheet (y, x1, x2, cross products, squares, normal equations)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AkzdwyHYSZDLsThLPh4WDM
</commit_message>
<xml_diff>
--- a/Tabel_10-6_Reaktor_Diferensial.xlsx
+++ b/Tabel_10-6_Reaktor_Diferensial.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Grafik" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Perhitungan" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="57">
   <si>
     <t xml:space="preserve">Tabel 10-6. Data dari Reaktor Diferensial (Hidrodemetilasi Toluena)</t>
   </si>
@@ -104,19 +105,121 @@
   </si>
   <si>
     <t xml:space="preserve">PT (atm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perhitungan Regresi Linear Berganda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model: -r'T = k·PH2·PT / (1 + KB·PB + KT·PT)  →  y = PH2·PT/(-r'T) = 1/k + (KB/k)·PB + (KT/k)·PT = a0 + a1·x1 + a2·x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-r'T dipakai sesuai tabel (nilai × 10^10). Metana tidak dimasukkan ke model karena Set A menunjukkan PM tidak berpengaruh. Teks hijau = link ke sheet Data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PH2
+(atm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT
+(atm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-r'T × 10^10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y = PH2·PT/(-rT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x1 = PB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x2 = PT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x1·y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x2·y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x1·x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x1²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x2²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Σ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Persamaan normal (Cramer):  [A]·[a0; a1; a2] = [b]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matriks A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vektor b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A0 (kolom 1 diganti b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1 (kolom 2 diganti b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2 (kolom 3 diganti b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hasil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">det A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a0 = 1/k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a1 = KB/k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a2 = KT/k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k (× 10^10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k (g mol/g kat·s·atm²)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KB (atm⁻¹)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KT (atm⁻¹)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0#"/>
     <numFmt numFmtId="167" formatCode="General"/>
+    <numFmt numFmtId="168" formatCode="0"/>
+    <numFmt numFmtId="169" formatCode="0.00000"/>
+    <numFmt numFmtId="170" formatCode="0.0000"/>
+    <numFmt numFmtId="171" formatCode="0.000000"/>
+    <numFmt numFmtId="172" formatCode="0.00"/>
+    <numFmt numFmtId="173" formatCode="0.00E+00"/>
+    <numFmt numFmtId="174" formatCode="0.000"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,8 +304,28 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -213,6 +336,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFDDE4EE"/>
         <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -265,7 +394,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -314,6 +443,58 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -343,7 +524,7 @@
       <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFF2CC"/>
       <rgbColor rgb="FFDDE4EE"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFE8833A"/>
@@ -521,11 +702,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="5499694"/>
-        <c:axId val="52315523"/>
+        <c:axId val="84838012"/>
+        <c:axId val="84891486"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="5499694"/>
+        <c:axId val="84838012"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -592,12 +773,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52315523"/>
+        <c:crossAx val="84891486"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="52315523"/>
+        <c:axId val="84891486"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -674,7 +855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5499694"/>
+        <c:crossAx val="84838012"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -925,11 +1106,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="36187160"/>
-        <c:axId val="56425051"/>
+        <c:axId val="36373273"/>
+        <c:axId val="1031734"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="36187160"/>
+        <c:axId val="36373273"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -996,12 +1177,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56425051"/>
+        <c:crossAx val="1031734"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="56425051"/>
+        <c:axId val="1031734"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1078,7 +1259,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36187160"/>
+        <c:crossAx val="36373273"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1271,11 +1452,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="27483764"/>
-        <c:axId val="2880661"/>
+        <c:axId val="33093098"/>
+        <c:axId val="31567085"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="27483764"/>
+        <c:axId val="33093098"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1342,12 +1523,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2880661"/>
+        <c:crossAx val="31567085"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2880661"/>
+        <c:axId val="31567085"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1424,7 +1605,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27483764"/>
+        <c:crossAx val="33093098"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1611,11 +1792,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="30684679"/>
-        <c:axId val="42570155"/>
+        <c:axId val="39088687"/>
+        <c:axId val="64981542"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="30684679"/>
+        <c:axId val="39088687"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1682,12 +1863,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42570155"/>
+        <c:crossAx val="64981542"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="42570155"/>
+        <c:axId val="64981542"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1764,7 +1945,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30684679"/>
+        <c:crossAx val="39088687"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2848,4 +3029,1200 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:L44"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="n">
+        <f aca="false">Data!B4</f>
+        <v>1</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <f aca="false">Data!E4</f>
+        <v>1</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <f aca="false">Data!D4</f>
+        <v>1</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <f aca="false">Data!C4</f>
+        <v>71</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <f aca="false">B6*C6/D6</f>
+        <v>0.0140845070422535</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <f aca="false">Data!G4</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <f aca="false">C6</f>
+        <v>1</v>
+      </c>
+      <c r="H6" s="14" t="n">
+        <f aca="false">F6*E6</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <f aca="false">G6*E6</f>
+        <v>0.0140845070422535</v>
+      </c>
+      <c r="J6" s="15" t="n">
+        <f aca="false">F6*G6</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="15" t="n">
+        <f aca="false">F6^2</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="15" t="n">
+        <f aca="false">G6^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="n">
+        <f aca="false">Data!B5</f>
+        <v>2</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <f aca="false">Data!E5</f>
+        <v>1</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <f aca="false">Data!D5</f>
+        <v>1</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <f aca="false">Data!C5</f>
+        <v>71.3</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <f aca="false">B7*C7/D7</f>
+        <v>0.0140252454417952</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <f aca="false">Data!G5</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <f aca="false">C7</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <f aca="false">F7*E7</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <f aca="false">G7*E7</f>
+        <v>0.0140252454417952</v>
+      </c>
+      <c r="J7" s="15" t="n">
+        <f aca="false">F7*G7</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="15" t="n">
+        <f aca="false">F7^2</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="15" t="n">
+        <f aca="false">G7^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="n">
+        <f aca="false">Data!B6</f>
+        <v>3</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <f aca="false">Data!E6</f>
+        <v>1</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <f aca="false">Data!D6</f>
+        <v>1</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <f aca="false">Data!C6</f>
+        <v>41.6</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <f aca="false">B8*C8/D8</f>
+        <v>0.0240384615384615</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <f aca="false">Data!G6</f>
+        <v>1</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <f aca="false">C8</f>
+        <v>1</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <f aca="false">F8*E8</f>
+        <v>0.0240384615384615</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <f aca="false">G8*E8</f>
+        <v>0.0240384615384615</v>
+      </c>
+      <c r="J8" s="15" t="n">
+        <f aca="false">F8*G8</f>
+        <v>1</v>
+      </c>
+      <c r="K8" s="15" t="n">
+        <f aca="false">F8^2</f>
+        <v>1</v>
+      </c>
+      <c r="L8" s="15" t="n">
+        <f aca="false">G8^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="n">
+        <f aca="false">Data!B7</f>
+        <v>4</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <f aca="false">Data!E7</f>
+        <v>1</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <f aca="false">Data!D7</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <f aca="false">Data!C7</f>
+        <v>19.7</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <f aca="false">B9*C9/D9</f>
+        <v>0.050761421319797</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <f aca="false">Data!G7</f>
+        <v>4</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <f aca="false">C9</f>
+        <v>1</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <f aca="false">F9*E9</f>
+        <v>0.203045685279188</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <f aca="false">G9*E9</f>
+        <v>0.050761421319797</v>
+      </c>
+      <c r="J9" s="15" t="n">
+        <f aca="false">F9*G9</f>
+        <v>4</v>
+      </c>
+      <c r="K9" s="15" t="n">
+        <f aca="false">F9^2</f>
+        <v>16</v>
+      </c>
+      <c r="L9" s="15" t="n">
+        <f aca="false">G9^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="n">
+        <f aca="false">Data!B8</f>
+        <v>5</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <f aca="false">Data!E8</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <f aca="false">Data!D8</f>
+        <v>1</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <f aca="false">Data!C8</f>
+        <v>42</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">B10*C10/D10</f>
+        <v>0.0238095238095238</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <f aca="false">Data!G8</f>
+        <v>1</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <f aca="false">C10</f>
+        <v>1</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <f aca="false">F10*E10</f>
+        <v>0.0238095238095238</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <f aca="false">G10*E10</f>
+        <v>0.0238095238095238</v>
+      </c>
+      <c r="J10" s="15" t="n">
+        <f aca="false">F10*G10</f>
+        <v>1</v>
+      </c>
+      <c r="K10" s="15" t="n">
+        <f aca="false">F10^2</f>
+        <v>1</v>
+      </c>
+      <c r="L10" s="15" t="n">
+        <f aca="false">G10^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="n">
+        <f aca="false">Data!B9</f>
+        <v>6</v>
+      </c>
+      <c r="B11" s="10" t="n">
+        <f aca="false">Data!E9</f>
+        <v>1</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <f aca="false">Data!D9</f>
+        <v>1</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <f aca="false">Data!C9</f>
+        <v>17.1</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <f aca="false">B11*C11/D11</f>
+        <v>0.0584795321637427</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <f aca="false">Data!G9</f>
+        <v>5</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <f aca="false">C11</f>
+        <v>1</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <f aca="false">F11*E11</f>
+        <v>0.292397660818713</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <f aca="false">G11*E11</f>
+        <v>0.0584795321637427</v>
+      </c>
+      <c r="J11" s="15" t="n">
+        <f aca="false">F11*G11</f>
+        <v>5</v>
+      </c>
+      <c r="K11" s="15" t="n">
+        <f aca="false">F11^2</f>
+        <v>25</v>
+      </c>
+      <c r="L11" s="15" t="n">
+        <f aca="false">G11^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="n">
+        <f aca="false">Data!B10</f>
+        <v>7</v>
+      </c>
+      <c r="B12" s="10" t="n">
+        <f aca="false">Data!E10</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <f aca="false">Data!D10</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <f aca="false">Data!C10</f>
+        <v>71.8</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <f aca="false">B12*C12/D12</f>
+        <v>0.0139275766016713</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <f aca="false">Data!G10</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <f aca="false">C12</f>
+        <v>1</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <f aca="false">F12*E12</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <f aca="false">G12*E12</f>
+        <v>0.0139275766016713</v>
+      </c>
+      <c r="J12" s="15" t="n">
+        <f aca="false">F12*G12</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="15" t="n">
+        <f aca="false">F12^2</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <f aca="false">G12^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="n">
+        <f aca="false">Data!B11</f>
+        <v>8</v>
+      </c>
+      <c r="B13" s="10" t="n">
+        <f aca="false">Data!E11</f>
+        <v>2</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <f aca="false">Data!D11</f>
+        <v>1</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <f aca="false">Data!C11</f>
+        <v>142</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <f aca="false">B13*C13/D13</f>
+        <v>0.0140845070422535</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <f aca="false">Data!G11</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <f aca="false">C13</f>
+        <v>1</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <f aca="false">F13*E13</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <f aca="false">G13*E13</f>
+        <v>0.0140845070422535</v>
+      </c>
+      <c r="J13" s="15" t="n">
+        <f aca="false">F13*G13</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="15" t="n">
+        <f aca="false">F13^2</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="15" t="n">
+        <f aca="false">G13^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="n">
+        <f aca="false">Data!B12</f>
+        <v>9</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <f aca="false">Data!E12</f>
+        <v>4</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <f aca="false">Data!D12</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <f aca="false">Data!C12</f>
+        <v>284</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <f aca="false">B14*C14/D14</f>
+        <v>0.0140845070422535</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <f aca="false">Data!G12</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <f aca="false">C14</f>
+        <v>1</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <f aca="false">F14*E14</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <f aca="false">G14*E14</f>
+        <v>0.0140845070422535</v>
+      </c>
+      <c r="J14" s="15" t="n">
+        <f aca="false">F14*G14</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="15" t="n">
+        <f aca="false">F14^2</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <f aca="false">G14^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="n">
+        <f aca="false">Data!B13</f>
+        <v>10</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <f aca="false">Data!E13</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <f aca="false">Data!D13</f>
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <f aca="false">Data!C13</f>
+        <v>47</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <f aca="false">B15*C15/D15</f>
+        <v>0.0106382978723404</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <f aca="false">Data!G13</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <f aca="false">C15</f>
+        <v>0.5</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <f aca="false">F15*E15</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <f aca="false">G15*E15</f>
+        <v>0.00531914893617021</v>
+      </c>
+      <c r="J15" s="15" t="n">
+        <f aca="false">F15*G15</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="15" t="n">
+        <f aca="false">F15^2</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <f aca="false">G15^2</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="n">
+        <f aca="false">Data!B14</f>
+        <v>11</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <f aca="false">Data!E14</f>
+        <v>1</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <f aca="false">Data!D14</f>
+        <v>1</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <f aca="false">Data!C14</f>
+        <v>71.3</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <f aca="false">B16*C16/D16</f>
+        <v>0.0140252454417952</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <f aca="false">Data!G14</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <f aca="false">C16</f>
+        <v>1</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <f aca="false">F16*E16</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="14" t="n">
+        <f aca="false">G16*E16</f>
+        <v>0.0140252454417952</v>
+      </c>
+      <c r="J16" s="15" t="n">
+        <f aca="false">F16*G16</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="15" t="n">
+        <f aca="false">F16^2</f>
+        <v>0</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <f aca="false">G16^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
+        <f aca="false">Data!B15</f>
+        <v>12</v>
+      </c>
+      <c r="B17" s="10" t="n">
+        <f aca="false">Data!E15</f>
+        <v>1</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <f aca="false">Data!D15</f>
+        <v>5</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <f aca="false">Data!C15</f>
+        <v>117</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <f aca="false">B17*C17/D17</f>
+        <v>0.0427350427350427</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <f aca="false">Data!G15</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <f aca="false">C17</f>
+        <v>5</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <f aca="false">F17*E17</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="14" t="n">
+        <f aca="false">G17*E17</f>
+        <v>0.213675213675214</v>
+      </c>
+      <c r="J17" s="15" t="n">
+        <f aca="false">F17*G17</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="15" t="n">
+        <f aca="false">F17^2</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <f aca="false">G17^2</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
+        <f aca="false">Data!B16</f>
+        <v>13</v>
+      </c>
+      <c r="B18" s="10" t="n">
+        <f aca="false">Data!E16</f>
+        <v>1</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <f aca="false">Data!D16</f>
+        <v>10</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <f aca="false">Data!C16</f>
+        <v>127</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <f aca="false">B18*C18/D18</f>
+        <v>0.078740157480315</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <f aca="false">Data!G16</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <f aca="false">C18</f>
+        <v>10</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <f aca="false">F18*E18</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="14" t="n">
+        <f aca="false">G18*E18</f>
+        <v>0.78740157480315</v>
+      </c>
+      <c r="J18" s="15" t="n">
+        <f aca="false">F18*G18</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="15" t="n">
+        <f aca="false">F18^2</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <f aca="false">G18^2</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
+        <f aca="false">Data!B17</f>
+        <v>14</v>
+      </c>
+      <c r="B19" s="10" t="n">
+        <f aca="false">Data!E17</f>
+        <v>1</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <f aca="false">Data!D17</f>
+        <v>15</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <f aca="false">Data!C17</f>
+        <v>131</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <f aca="false">B19*C19/D19</f>
+        <v>0.114503816793893</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <f aca="false">Data!G17</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <f aca="false">C19</f>
+        <v>15</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <f aca="false">F19*E19</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="14" t="n">
+        <f aca="false">G19*E19</f>
+        <v>1.7175572519084</v>
+      </c>
+      <c r="J19" s="15" t="n">
+        <f aca="false">F19*G19</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="15" t="n">
+        <f aca="false">F19^2</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="15" t="n">
+        <f aca="false">G19^2</f>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="n">
+        <f aca="false">Data!B18</f>
+        <v>15</v>
+      </c>
+      <c r="B20" s="10" t="n">
+        <f aca="false">Data!E18</f>
+        <v>1</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <f aca="false">Data!D18</f>
+        <v>20</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <f aca="false">Data!C18</f>
+        <v>133</v>
+      </c>
+      <c r="E20" s="14" t="n">
+        <f aca="false">B20*C20/D20</f>
+        <v>0.150375939849624</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <f aca="false">Data!G18</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <f aca="false">C20</f>
+        <v>20</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <f aca="false">F20*E20</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="14" t="n">
+        <f aca="false">G20*E20</f>
+        <v>3.00751879699248</v>
+      </c>
+      <c r="J20" s="15" t="n">
+        <f aca="false">F20*G20</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="15" t="n">
+        <f aca="false">F20^2</f>
+        <v>0</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <f aca="false">G20^2</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="n">
+        <f aca="false">Data!B19</f>
+        <v>16</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <f aca="false">Data!E19</f>
+        <v>1</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <f aca="false">Data!D19</f>
+        <v>1</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <f aca="false">Data!C19</f>
+        <v>41.8</v>
+      </c>
+      <c r="E21" s="14" t="n">
+        <f aca="false">B21*C21/D21</f>
+        <v>0.0239234449760766</v>
+      </c>
+      <c r="F21" s="10" t="n">
+        <f aca="false">Data!G19</f>
+        <v>1</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <f aca="false">C21</f>
+        <v>1</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <f aca="false">F21*E21</f>
+        <v>0.0239234449760766</v>
+      </c>
+      <c r="I21" s="14" t="n">
+        <f aca="false">G21*E21</f>
+        <v>0.0239234449760766</v>
+      </c>
+      <c r="J21" s="15" t="n">
+        <f aca="false">F21*G21</f>
+        <v>1</v>
+      </c>
+      <c r="K21" s="15" t="n">
+        <f aca="false">F21^2</f>
+        <v>1</v>
+      </c>
+      <c r="L21" s="15" t="n">
+        <f aca="false">G21^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <f aca="false">COUNT(E6:E21)</f>
+        <v>16</v>
+      </c>
+      <c r="E22" s="16" t="n">
+        <f aca="false">SUM(E6:E21)</f>
+        <v>0.662237227150839</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <f aca="false">SUM(F6:F21)</f>
+        <v>12</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <f aca="false">SUM(G6:G21)</f>
+        <v>61.5</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <f aca="false">SUM(H6:H21)</f>
+        <v>0.567214776421963</v>
+      </c>
+      <c r="I22" s="16" t="n">
+        <f aca="false">SUM(I6:I21)</f>
+        <v>5.99671595873504</v>
+      </c>
+      <c r="J22" s="17" t="n">
+        <f aca="false">SUM(J6:J21)</f>
+        <v>12</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <f aca="false">SUM(K6:K21)</f>
+        <v>44</v>
+      </c>
+      <c r="L22" s="17" t="n">
+        <f aca="false">SUM(L6:L21)</f>
+        <v>761.25</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="19" t="n">
+        <f aca="false">$C$22</f>
+        <v>16</v>
+      </c>
+      <c r="C27" s="19" t="n">
+        <f aca="false">$F$22</f>
+        <v>12</v>
+      </c>
+      <c r="D27" s="19" t="n">
+        <f aca="false">$G$22</f>
+        <v>61.5</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <f aca="false">$E$22</f>
+        <v>0.662237227150839</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="19" t="n">
+        <f aca="false">$F$22</f>
+        <v>12</v>
+      </c>
+      <c r="C28" s="19" t="n">
+        <f aca="false">$K$22</f>
+        <v>44</v>
+      </c>
+      <c r="D28" s="19" t="n">
+        <f aca="false">$J$22</f>
+        <v>12</v>
+      </c>
+      <c r="F28" s="19" t="n">
+        <f aca="false">$H$22</f>
+        <v>0.567214776421963</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="19" t="n">
+        <f aca="false">$G$22</f>
+        <v>61.5</v>
+      </c>
+      <c r="C29" s="19" t="n">
+        <f aca="false">$J$22</f>
+        <v>12</v>
+      </c>
+      <c r="D29" s="19" t="n">
+        <f aca="false">$L$22</f>
+        <v>761.25</v>
+      </c>
+      <c r="F29" s="19" t="n">
+        <f aca="false">$I$22</f>
+        <v>5.99671595873504</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="J31" s="18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="19" t="n">
+        <f aca="false">$E$22</f>
+        <v>0.662237227150839</v>
+      </c>
+      <c r="C32" s="19" t="n">
+        <f aca="false">$F$22</f>
+        <v>12</v>
+      </c>
+      <c r="D32" s="19" t="n">
+        <f aca="false">$G$22</f>
+        <v>61.5</v>
+      </c>
+      <c r="F32" s="19" t="n">
+        <f aca="false">$C$22</f>
+        <v>16</v>
+      </c>
+      <c r="G32" s="19" t="n">
+        <f aca="false">$E$22</f>
+        <v>0.662237227150839</v>
+      </c>
+      <c r="H32" s="19" t="n">
+        <f aca="false">$G$22</f>
+        <v>61.5</v>
+      </c>
+      <c r="J32" s="19" t="n">
+        <f aca="false">$C$22</f>
+        <v>16</v>
+      </c>
+      <c r="K32" s="19" t="n">
+        <f aca="false">$F$22</f>
+        <v>12</v>
+      </c>
+      <c r="L32" s="19" t="n">
+        <f aca="false">$E$22</f>
+        <v>0.662237227150839</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="19" t="n">
+        <f aca="false">$H$22</f>
+        <v>0.567214776421963</v>
+      </c>
+      <c r="C33" s="19" t="n">
+        <f aca="false">$K$22</f>
+        <v>44</v>
+      </c>
+      <c r="D33" s="19" t="n">
+        <f aca="false">$J$22</f>
+        <v>12</v>
+      </c>
+      <c r="F33" s="19" t="n">
+        <f aca="false">$F$22</f>
+        <v>12</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <f aca="false">$H$22</f>
+        <v>0.567214776421963</v>
+      </c>
+      <c r="H33" s="19" t="n">
+        <f aca="false">$J$22</f>
+        <v>12</v>
+      </c>
+      <c r="J33" s="19" t="n">
+        <f aca="false">$F$22</f>
+        <v>12</v>
+      </c>
+      <c r="K33" s="19" t="n">
+        <f aca="false">$K$22</f>
+        <v>44</v>
+      </c>
+      <c r="L33" s="19" t="n">
+        <f aca="false">$H$22</f>
+        <v>0.567214776421963</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="19" t="n">
+        <f aca="false">$I$22</f>
+        <v>5.99671595873504</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <f aca="false">$J$22</f>
+        <v>12</v>
+      </c>
+      <c r="D34" s="19" t="n">
+        <f aca="false">$L$22</f>
+        <v>761.25</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <f aca="false">$G$22</f>
+        <v>61.5</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <f aca="false">$I$22</f>
+        <v>5.99671595873504</v>
+      </c>
+      <c r="H34" s="19" t="n">
+        <f aca="false">$L$22</f>
+        <v>761.25</v>
+      </c>
+      <c r="J34" s="19" t="n">
+        <f aca="false">$G$22</f>
+        <v>61.5</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <f aca="false">$J$22</f>
+        <v>12</v>
+      </c>
+      <c r="L34" s="19" t="n">
+        <f aca="false">$I$22</f>
+        <v>5.99671595873504</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="19" t="n">
+        <f aca="false">MDETERM(B27:D29)</f>
+        <v>275289</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38" s="21" t="n">
+        <f aca="false">MDETERM(B32:D34)/C37</f>
+        <v>0.00711900947300202</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="21" t="n">
+        <f aca="false">MDETERM(F32:H34)/C37</f>
+        <v>0.00899683171423948</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C40" s="21" t="n">
+        <f aca="false">MDETERM(J32:L34)/C37</f>
+        <v>0.00716050560995013</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C41" s="22" t="n">
+        <f aca="false">1/C38</f>
+        <v>140.468980100726</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C42" s="23" t="n">
+        <f aca="false">C41*0.0000000001</f>
+        <v>1.40468980100726E-008</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C43" s="24" t="n">
+        <f aca="false">C39/C38</f>
+        <v>1.26377577503709</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C44" s="24" t="n">
+        <f aca="false">C40/C38</f>
+        <v>1.00582892003522</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add model predictions, R², and regression plots for y = a0 + a1x1 + a2x2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AkzdwyHYSZDLsThLPh4WDM
</commit_message>
<xml_diff>
--- a/Tabel_10-6_Reaktor_Diferensial.xlsx
+++ b/Tabel_10-6_Reaktor_Diferensial.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Grafik" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Perhitungan" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Plot Regresi" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="71">
   <si>
     <t xml:space="preserve">Tabel 10-6. Data dari Reaktor Diferensial (Hidrodemetilasi Toluena)</t>
   </si>
@@ -151,6 +152,13 @@
     <t xml:space="preserve">x2²</t>
   </si>
   <si>
+    <t xml:space="preserve">ŷ = a0 + a1·x1 + a2·x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residual
+y − ŷ</t>
+  </si>
+  <si>
     <t xml:space="preserve">Σ</t>
   </si>
   <si>
@@ -200,13 +208,49 @@
   </si>
   <si>
     <t xml:space="preserve">KT (atm⁻¹)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSE = Σ(y − ŷ)²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SST = Σ(y − ȳ)²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R² = 1 − SSE/SST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Persamaan hasil regresi:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plot Regresi: y = a0 + a1·x1 + a2·x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabel bantu mengambil nilai dari sheet Perhitungan (teks hijau = link antar-sheet).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) y data vs ŷ model (semua run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ŷ model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garis y = ŷ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2) y vs x2 = PT (x1 = PB = 0, Set D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3) y vs x1 = PB (x2 = PT = 1, PM = 0)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0#"/>
@@ -218,8 +262,9 @@
     <numFmt numFmtId="172" formatCode="0.00"/>
     <numFmt numFmtId="173" formatCode="0.00E+00"/>
     <numFmt numFmtId="174" formatCode="0.000"/>
+    <numFmt numFmtId="175" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -312,6 +357,12 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="9"/>
       <name val="Arial"/>
@@ -319,7 +370,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -394,7 +445,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -459,6 +510,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="169" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -467,19 +522,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -492,6 +547,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="174" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -552,7 +627,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF888888"/>
       <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -702,11 +777,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="84838012"/>
-        <c:axId val="84891486"/>
+        <c:axId val="1326939"/>
+        <c:axId val="25140594"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="84838012"/>
+        <c:axId val="1326939"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -773,12 +848,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84891486"/>
+        <c:crossAx val="25140594"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="84891486"/>
+        <c:axId val="25140594"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -855,7 +930,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84838012"/>
+        <c:crossAx val="1326939"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1106,11 +1181,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="36373273"/>
-        <c:axId val="1031734"/>
+        <c:axId val="11637463"/>
+        <c:axId val="47213593"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="36373273"/>
+        <c:axId val="11637463"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1177,12 +1252,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1031734"/>
+        <c:crossAx val="47213593"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1031734"/>
+        <c:axId val="47213593"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1259,7 +1334,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36373273"/>
+        <c:crossAx val="11637463"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1452,11 +1527,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="33093098"/>
-        <c:axId val="31567085"/>
+        <c:axId val="82038874"/>
+        <c:axId val="50306150"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="33093098"/>
+        <c:axId val="82038874"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1523,12 +1598,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31567085"/>
+        <c:crossAx val="50306150"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="31567085"/>
+        <c:axId val="50306150"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1605,7 +1680,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33093098"/>
+        <c:crossAx val="82038874"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1792,11 +1867,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="39088687"/>
-        <c:axId val="64981542"/>
+        <c:axId val="80747851"/>
+        <c:axId val="81129484"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="39088687"/>
+        <c:axId val="80747851"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1863,12 +1938,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64981542"/>
+        <c:crossAx val="81129484"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="64981542"/>
+        <c:axId val="81129484"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1945,7 +2020,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39088687"/>
+        <c:crossAx val="80747851"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1956,6 +2031,1429 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>y data vs ŷ model (parity plot)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Data (Run 1–16)"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Data (Run 1–16)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2a6fdb"/>
+            </a:solidFill>
+            <a:ln w="47520">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2a6fdb"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$B$7:$B$22</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0232763467971916</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0502668419399101</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.0232763467971916</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.0592636736541496</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.0106992622779771</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.0429215375227527</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.0787240655725033</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.114526593622254</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.150329121672005</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.0232763467971916</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$C$7:$C$22</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>0.0140845070422535</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0140252454417952</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0240384615384615</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.050761421319797</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.0238095238095238</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.0584795321637427</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.0139275766016713</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.0140845070422535</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.0140845070422535</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.0106382978723404</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.0140252454417952</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.0427350427350427</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.078740157480315</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.114503816793893</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.150375939849624</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.0239234449760766</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Garis y = ŷ"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Garis y = ŷ</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="888888"/>
+            </a:solidFill>
+            <a:ln w="21960">
+              <a:solidFill>
+                <a:srgbClr val="888888"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$B$25:$B$26</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.157894736842105</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$C$25:$C$26</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.157894736842105</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:axId val="12120149"/>
+        <c:axId val="68585837"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="12120149"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>ŷ = a0 + a1·x1 + a2·x2</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="68585837"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="68585837"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>y = PH2·PT/(-r'T)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="12120149"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>y vs x2 (PB = 0)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Data Set D (Run 10–15)"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Data Set D (Run 10–15)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2a6fdb"/>
+            </a:solidFill>
+            <a:ln w="47520">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2a6fdb"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$A$31:$A$36</c:f>
+              <c:numCache>
+                <c:formatCode>0.0#</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$B$31:$B$36</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.0106382978723404</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0140252454417952</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0427350427350427</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.078740157480315</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.114503816793893</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.150375939849624</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Model: ŷ = a0 + a2·x2"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Model: ŷ = a0 + a2·x2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="e8833a"/>
+            </a:solidFill>
+            <a:ln w="21960">
+              <a:solidFill>
+                <a:srgbClr val="e8833a"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$A$31:$A$36</c:f>
+              <c:numCache>
+                <c:formatCode>0.0#</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$C$31:$C$36</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.0106992622779771</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0429215375227527</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0787240655725033</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.114526593622254</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.150329121672005</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:axId val="30879269"/>
+        <c:axId val="95176001"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="30879269"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>x2 = PT (atm)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.0#" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="95176001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="95176001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>y = PH2·PT/(-r'T)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="30879269"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>y vs x1 (PT = 1)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Data Run 7, 3, 4, 6"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Data Run 7, 3, 4, 6</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2a6fdb"/>
+            </a:solidFill>
+            <a:ln w="47520">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2a6fdb"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$A$41:$A$44</c:f>
+              <c:numCache>
+                <c:formatCode>0.0#</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$B$41:$B$44</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.0139275766016713</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0240384615384615</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.050761421319797</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0584795321637427</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Model: ŷ = (a0 + a2) + a1·x1"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Model: ŷ = (a0 + a2) + a1·x1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="e8833a"/>
+            </a:solidFill>
+            <a:ln w="21960">
+              <a:solidFill>
+                <a:srgbClr val="e8833a"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$A$41:$A$44</c:f>
+              <c:numCache>
+                <c:formatCode>0.0#</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Plot Regresi'!$C$41:$C$44</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.0142795150829522</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0232763467971916</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0502668419399101</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0592636736541496</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:axId val="9329568"/>
+        <c:axId val="33116245"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="9329568"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>x1 = PB (atm)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.0#" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="33116245"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="33116245"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>y = PH2·PT/(-r'T)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="9329568"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
@@ -2090,6 +3588,101 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>507600</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>187560</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="3008160" y="762120"/>
+        <a:ext cx="5399640" cy="3059640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>507600</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>187560</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="3008160" y="4381560"/>
+        <a:ext cx="5399640" cy="3059640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>507600</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>187560</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="3008160" y="8001000"/>
+        <a:ext cx="5399640" cy="3059640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3036,7 +4629,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -3048,6 +4641,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,6 +4697,12 @@
       <c r="L5" s="2" t="s">
         <v>39</v>
       </c>
+      <c r="M5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="n">
@@ -3151,6 +4752,14 @@
       <c r="L6" s="15" t="n">
         <f aca="false">G6^2</f>
         <v>1</v>
+      </c>
+      <c r="M6" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F6+$C$40*G6</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="N6" s="16" t="n">
+        <f aca="false">E6-M6</f>
+        <v>-0.000195008040698632</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3202,6 +4811,14 @@
         <f aca="false">G7^2</f>
         <v>1</v>
       </c>
+      <c r="M7" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F7+$C$40*G7</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="N7" s="16" t="n">
+        <f aca="false">E7-M7</f>
+        <v>-0.000254269641156921</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="n">
@@ -3252,6 +4869,14 @@
         <f aca="false">G8^2</f>
         <v>1</v>
       </c>
+      <c r="M8" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F8+$C$40*G8</f>
+        <v>0.0232763467971916</v>
+      </c>
+      <c r="N8" s="16" t="n">
+        <f aca="false">E8-M8</f>
+        <v>0.000762114741269901</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="n">
@@ -3302,6 +4927,14 @@
         <f aca="false">G9^2</f>
         <v>1</v>
       </c>
+      <c r="M9" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F9+$C$40*G9</f>
+        <v>0.0502668419399101</v>
+      </c>
+      <c r="N9" s="16" t="n">
+        <f aca="false">E9-M9</f>
+        <v>0.000494579379886874</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="n">
@@ -3352,6 +4985,14 @@
         <f aca="false">G10^2</f>
         <v>1</v>
       </c>
+      <c r="M10" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F10+$C$40*G10</f>
+        <v>0.0232763467971916</v>
+      </c>
+      <c r="N10" s="16" t="n">
+        <f aca="false">E10-M10</f>
+        <v>0.000533177012332173</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="n">
@@ -3402,6 +5043,14 @@
         <f aca="false">G11^2</f>
         <v>1</v>
       </c>
+      <c r="M11" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F11+$C$40*G11</f>
+        <v>0.0592636736541496</v>
+      </c>
+      <c r="N11" s="16" t="n">
+        <f aca="false">E11-M11</f>
+        <v>-0.000784141490406877</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="n">
@@ -3452,6 +5101,14 @@
         <f aca="false">G12^2</f>
         <v>1</v>
       </c>
+      <c r="M12" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F12+$C$40*G12</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="N12" s="16" t="n">
+        <f aca="false">E12-M12</f>
+        <v>-0.000351938481280843</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="n">
@@ -3502,6 +5159,14 @@
         <f aca="false">G13^2</f>
         <v>1</v>
       </c>
+      <c r="M13" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F13+$C$40*G13</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="N13" s="16" t="n">
+        <f aca="false">E13-M13</f>
+        <v>-0.000195008040698632</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="n">
@@ -3552,6 +5217,14 @@
         <f aca="false">G14^2</f>
         <v>1</v>
       </c>
+      <c r="M14" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F14+$C$40*G14</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="N14" s="16" t="n">
+        <f aca="false">E14-M14</f>
+        <v>-0.000195008040698632</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="n">
@@ -3602,6 +5275,14 @@
         <f aca="false">G15^2</f>
         <v>0.25</v>
       </c>
+      <c r="M15" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F15+$C$40*G15</f>
+        <v>0.0106992622779771</v>
+      </c>
+      <c r="N15" s="16" t="n">
+        <f aca="false">E15-M15</f>
+        <v>-6.09644056366616E-005</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="n">
@@ -3652,6 +5333,14 @@
         <f aca="false">G16^2</f>
         <v>1</v>
       </c>
+      <c r="M16" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F16+$C$40*G16</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="N16" s="16" t="n">
+        <f aca="false">E16-M16</f>
+        <v>-0.000254269641156921</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="n">
@@ -3702,6 +5391,14 @@
         <f aca="false">G17^2</f>
         <v>25</v>
       </c>
+      <c r="M17" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F17+$C$40*G17</f>
+        <v>0.0429215375227527</v>
+      </c>
+      <c r="N17" s="16" t="n">
+        <f aca="false">E17-M17</f>
+        <v>-0.000186494787709941</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="n">
@@ -3752,6 +5449,14 @@
         <f aca="false">G18^2</f>
         <v>100</v>
       </c>
+      <c r="M18" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F18+$C$40*G18</f>
+        <v>0.0787240655725033</v>
+      </c>
+      <c r="N18" s="16" t="n">
+        <f aca="false">E18-M18</f>
+        <v>1.60919078116273E-005</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="n">
@@ -3802,6 +5507,14 @@
         <f aca="false">G19^2</f>
         <v>225</v>
       </c>
+      <c r="M19" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F19+$C$40*G19</f>
+        <v>0.114526593622254</v>
+      </c>
+      <c r="N19" s="16" t="n">
+        <f aca="false">E19-M19</f>
+        <v>-2.27768283608681E-005</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="n">
@@ -3852,6 +5565,14 @@
         <f aca="false">G20^2</f>
         <v>400</v>
       </c>
+      <c r="M20" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F20+$C$40*G20</f>
+        <v>0.150329121672005</v>
+      </c>
+      <c r="N20" s="16" t="n">
+        <f aca="false">E20-M20</f>
+        <v>4.68181776194232E-005</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="n">
@@ -3902,318 +5623,368 @@
         <f aca="false">G21^2</f>
         <v>1</v>
       </c>
+      <c r="M21" s="16" t="n">
+        <f aca="false">$C$38+$C$39*F21+$C$40*G21</f>
+        <v>0.0232763467971916</v>
+      </c>
+      <c r="N21" s="16" t="n">
+        <f aca="false">E21-M21</f>
+        <v>0.00064709817888492</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C22" s="7" t="n">
         <f aca="false">COUNT(E6:E21)</f>
         <v>16</v>
       </c>
-      <c r="E22" s="16" t="n">
+      <c r="E22" s="17" t="n">
         <f aca="false">SUM(E6:E21)</f>
         <v>0.662237227150839</v>
       </c>
-      <c r="F22" s="17" t="n">
+      <c r="F22" s="18" t="n">
         <f aca="false">SUM(F6:F21)</f>
         <v>12</v>
       </c>
-      <c r="G22" s="17" t="n">
+      <c r="G22" s="18" t="n">
         <f aca="false">SUM(G6:G21)</f>
         <v>61.5</v>
       </c>
-      <c r="H22" s="16" t="n">
+      <c r="H22" s="17" t="n">
         <f aca="false">SUM(H6:H21)</f>
         <v>0.567214776421963</v>
       </c>
-      <c r="I22" s="16" t="n">
+      <c r="I22" s="17" t="n">
         <f aca="false">SUM(I6:I21)</f>
         <v>5.99671595873504</v>
       </c>
-      <c r="J22" s="17" t="n">
+      <c r="J22" s="18" t="n">
         <f aca="false">SUM(J6:J21)</f>
         <v>12</v>
       </c>
-      <c r="K22" s="17" t="n">
+      <c r="K22" s="18" t="n">
         <f aca="false">SUM(K6:K21)</f>
         <v>44</v>
       </c>
-      <c r="L22" s="17" t="n">
+      <c r="L22" s="18" t="n">
         <f aca="false">SUM(L6:L21)</f>
         <v>761.25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>44</v>
+      <c r="B26" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="19" t="n">
+      <c r="B27" s="20" t="n">
         <f aca="false">$C$22</f>
         <v>16</v>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="20" t="n">
         <f aca="false">$F$22</f>
         <v>12</v>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D27" s="20" t="n">
         <f aca="false">$G$22</f>
         <v>61.5</v>
       </c>
-      <c r="F27" s="19" t="n">
+      <c r="F27" s="20" t="n">
         <f aca="false">$E$22</f>
         <v>0.662237227150839</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="19" t="n">
+      <c r="B28" s="20" t="n">
         <f aca="false">$F$22</f>
         <v>12</v>
       </c>
-      <c r="C28" s="19" t="n">
+      <c r="C28" s="20" t="n">
         <f aca="false">$K$22</f>
         <v>44</v>
       </c>
-      <c r="D28" s="19" t="n">
+      <c r="D28" s="20" t="n">
         <f aca="false">$J$22</f>
         <v>12</v>
       </c>
-      <c r="F28" s="19" t="n">
+      <c r="F28" s="20" t="n">
         <f aca="false">$H$22</f>
         <v>0.567214776421963</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="19" t="n">
+      <c r="B29" s="20" t="n">
         <f aca="false">$G$22</f>
         <v>61.5</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="20" t="n">
         <f aca="false">$J$22</f>
         <v>12</v>
       </c>
-      <c r="D29" s="19" t="n">
+      <c r="D29" s="20" t="n">
         <f aca="false">$L$22</f>
         <v>761.25</v>
       </c>
-      <c r="F29" s="19" t="n">
+      <c r="F29" s="20" t="n">
         <f aca="false">$I$22</f>
         <v>5.99671595873504</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="F31" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="J31" s="18" t="s">
+      <c r="B31" s="19" t="s">
         <v>47</v>
       </c>
+      <c r="F31" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="J31" s="19" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="19" t="n">
+      <c r="B32" s="20" t="n">
         <f aca="false">$E$22</f>
         <v>0.662237227150839</v>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C32" s="20" t="n">
         <f aca="false">$F$22</f>
         <v>12</v>
       </c>
-      <c r="D32" s="19" t="n">
+      <c r="D32" s="20" t="n">
         <f aca="false">$G$22</f>
         <v>61.5</v>
       </c>
-      <c r="F32" s="19" t="n">
+      <c r="F32" s="20" t="n">
         <f aca="false">$C$22</f>
         <v>16</v>
       </c>
-      <c r="G32" s="19" t="n">
+      <c r="G32" s="20" t="n">
         <f aca="false">$E$22</f>
         <v>0.662237227150839</v>
       </c>
-      <c r="H32" s="19" t="n">
+      <c r="H32" s="20" t="n">
         <f aca="false">$G$22</f>
         <v>61.5</v>
       </c>
-      <c r="J32" s="19" t="n">
+      <c r="J32" s="20" t="n">
         <f aca="false">$C$22</f>
         <v>16</v>
       </c>
-      <c r="K32" s="19" t="n">
+      <c r="K32" s="20" t="n">
         <f aca="false">$F$22</f>
         <v>12</v>
       </c>
-      <c r="L32" s="19" t="n">
+      <c r="L32" s="20" t="n">
         <f aca="false">$E$22</f>
         <v>0.662237227150839</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="19" t="n">
+      <c r="B33" s="20" t="n">
         <f aca="false">$H$22</f>
         <v>0.567214776421963</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C33" s="20" t="n">
         <f aca="false">$K$22</f>
         <v>44</v>
       </c>
-      <c r="D33" s="19" t="n">
+      <c r="D33" s="20" t="n">
         <f aca="false">$J$22</f>
         <v>12</v>
       </c>
-      <c r="F33" s="19" t="n">
+      <c r="F33" s="20" t="n">
         <f aca="false">$F$22</f>
         <v>12</v>
       </c>
-      <c r="G33" s="19" t="n">
+      <c r="G33" s="20" t="n">
         <f aca="false">$H$22</f>
         <v>0.567214776421963</v>
       </c>
-      <c r="H33" s="19" t="n">
+      <c r="H33" s="20" t="n">
         <f aca="false">$J$22</f>
         <v>12</v>
       </c>
-      <c r="J33" s="19" t="n">
+      <c r="J33" s="20" t="n">
         <f aca="false">$F$22</f>
         <v>12</v>
       </c>
-      <c r="K33" s="19" t="n">
+      <c r="K33" s="20" t="n">
         <f aca="false">$K$22</f>
         <v>44</v>
       </c>
-      <c r="L33" s="19" t="n">
+      <c r="L33" s="20" t="n">
         <f aca="false">$H$22</f>
         <v>0.567214776421963</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="19" t="n">
+      <c r="B34" s="20" t="n">
         <f aca="false">$I$22</f>
         <v>5.99671595873504</v>
       </c>
-      <c r="C34" s="19" t="n">
+      <c r="C34" s="20" t="n">
         <f aca="false">$J$22</f>
         <v>12</v>
       </c>
-      <c r="D34" s="19" t="n">
+      <c r="D34" s="20" t="n">
         <f aca="false">$L$22</f>
         <v>761.25</v>
       </c>
-      <c r="F34" s="19" t="n">
+      <c r="F34" s="20" t="n">
         <f aca="false">$G$22</f>
         <v>61.5</v>
       </c>
-      <c r="G34" s="19" t="n">
+      <c r="G34" s="20" t="n">
         <f aca="false">$I$22</f>
         <v>5.99671595873504</v>
       </c>
-      <c r="H34" s="19" t="n">
+      <c r="H34" s="20" t="n">
         <f aca="false">$L$22</f>
         <v>761.25</v>
       </c>
-      <c r="J34" s="19" t="n">
+      <c r="J34" s="20" t="n">
         <f aca="false">$G$22</f>
         <v>61.5</v>
       </c>
-      <c r="K34" s="19" t="n">
+      <c r="K34" s="20" t="n">
         <f aca="false">$J$22</f>
         <v>12</v>
       </c>
-      <c r="L34" s="19" t="n">
+      <c r="L34" s="20" t="n">
         <f aca="false">$I$22</f>
         <v>5.99671595873504</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="C37" s="19" t="n">
+      <c r="A37" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C37" s="20" t="n">
         <f aca="false">MDETERM(B27:D29)</f>
         <v>275289</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="C38" s="21" t="n">
+      <c r="A38" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C38" s="22" t="n">
         <f aca="false">MDETERM(B32:D34)/C37</f>
         <v>0.00711900947300202</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C39" s="21" t="n">
+      <c r="A39" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C39" s="22" t="n">
         <f aca="false">MDETERM(F32:H34)/C37</f>
         <v>0.00899683171423948</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C40" s="21" t="n">
+      <c r="A40" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C40" s="22" t="n">
         <f aca="false">MDETERM(J32:L34)/C37</f>
         <v>0.00716050560995013</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="C41" s="22" t="n">
+        <v>55</v>
+      </c>
+      <c r="C41" s="23" t="n">
         <f aca="false">1/C38</f>
         <v>140.468980100726</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C42" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="C42" s="24" t="n">
         <f aca="false">C41*0.0000000001</f>
         <v>1.40468980100726E-008</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="C43" s="24" t="n">
+        <v>57</v>
+      </c>
+      <c r="C43" s="25" t="n">
         <f aca="false">C39/C38</f>
         <v>1.26377577503709</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" s="24" t="n">
+        <v>58</v>
+      </c>
+      <c r="C44" s="25" t="n">
         <f aca="false">C40/C38</f>
         <v>1.00582892003522</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C45" s="26" t="n">
+        <f aca="false">SUMSQ(N6:N21)</f>
+        <v>2.5520371414495E-006</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C46" s="26" t="n">
+        <f aca="false">DEVSQ(E6:E21)</f>
+        <v>0.0253497952196739</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C47" s="27" t="n">
+        <f aca="false">1-C45/C46</f>
+        <v>0.999899327110167</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C49" s="7" t="str">
+        <f aca="false">"y = "&amp;TEXT($C$38,"0.000000")&amp;" + "&amp;TEXT($C$39,"0.000000")&amp;"·x1 + "&amp;TEXT($C$40,"0.000000")&amp;"·x2"</f>
+        <v>y = 0.007119 + 0.008997·x1 + 0.007161·x2</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C50" s="7" t="str">
+        <f aca="false">"-r'T = "&amp;TEXT(C42,"0.00E+00")&amp;"·PH2·PT / (1 + "&amp;TEXT(C43,"0.000")&amp;"·PB + "&amp;TEXT(C44,"0.000")&amp;"·PT)"</f>
+        <v>-r'T = 1.40E-08·PH2·PT / (1 + 1.264·PB + 1.006·PT)</v>
       </c>
     </row>
   </sheetData>
@@ -4225,4 +5996,481 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C44"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="28" t="str">
+        <f aca="false">"a0 = "&amp;TEXT(Perhitungan!$C$38,"0.000000")&amp;"   a1 = "&amp;TEXT(Perhitungan!$C$39,"0.000000")&amp;"   a2 = "&amp;TEXT(Perhitungan!$C$40,"0.000000")&amp;"   R² = "&amp;TEXT(Perhitungan!C47,"0.0000")</f>
+        <v>a0 = 0.007119   a1 = 0.008997   a2 = 0.007161   R² = 0.9999</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="n">
+        <f aca="false">Perhitungan!A6</f>
+        <v>1</v>
+      </c>
+      <c r="B7" s="30" t="n">
+        <f aca="false">Perhitungan!M6</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="C7" s="30" t="n">
+        <f aca="false">Perhitungan!E6</f>
+        <v>0.0140845070422535</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="n">
+        <f aca="false">Perhitungan!A7</f>
+        <v>2</v>
+      </c>
+      <c r="B8" s="30" t="n">
+        <f aca="false">Perhitungan!M7</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="C8" s="30" t="n">
+        <f aca="false">Perhitungan!E7</f>
+        <v>0.0140252454417952</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="n">
+        <f aca="false">Perhitungan!A8</f>
+        <v>3</v>
+      </c>
+      <c r="B9" s="30" t="n">
+        <f aca="false">Perhitungan!M8</f>
+        <v>0.0232763467971916</v>
+      </c>
+      <c r="C9" s="30" t="n">
+        <f aca="false">Perhitungan!E8</f>
+        <v>0.0240384615384615</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="n">
+        <f aca="false">Perhitungan!A9</f>
+        <v>4</v>
+      </c>
+      <c r="B10" s="30" t="n">
+        <f aca="false">Perhitungan!M9</f>
+        <v>0.0502668419399101</v>
+      </c>
+      <c r="C10" s="30" t="n">
+        <f aca="false">Perhitungan!E9</f>
+        <v>0.050761421319797</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="n">
+        <f aca="false">Perhitungan!A10</f>
+        <v>5</v>
+      </c>
+      <c r="B11" s="30" t="n">
+        <f aca="false">Perhitungan!M10</f>
+        <v>0.0232763467971916</v>
+      </c>
+      <c r="C11" s="30" t="n">
+        <f aca="false">Perhitungan!E10</f>
+        <v>0.0238095238095238</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="n">
+        <f aca="false">Perhitungan!A11</f>
+        <v>6</v>
+      </c>
+      <c r="B12" s="30" t="n">
+        <f aca="false">Perhitungan!M11</f>
+        <v>0.0592636736541496</v>
+      </c>
+      <c r="C12" s="30" t="n">
+        <f aca="false">Perhitungan!E11</f>
+        <v>0.0584795321637427</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="n">
+        <f aca="false">Perhitungan!A12</f>
+        <v>7</v>
+      </c>
+      <c r="B13" s="30" t="n">
+        <f aca="false">Perhitungan!M12</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="C13" s="30" t="n">
+        <f aca="false">Perhitungan!E12</f>
+        <v>0.0139275766016713</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="n">
+        <f aca="false">Perhitungan!A13</f>
+        <v>8</v>
+      </c>
+      <c r="B14" s="30" t="n">
+        <f aca="false">Perhitungan!M13</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="C14" s="30" t="n">
+        <f aca="false">Perhitungan!E13</f>
+        <v>0.0140845070422535</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="n">
+        <f aca="false">Perhitungan!A14</f>
+        <v>9</v>
+      </c>
+      <c r="B15" s="30" t="n">
+        <f aca="false">Perhitungan!M14</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <f aca="false">Perhitungan!E14</f>
+        <v>0.0140845070422535</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="n">
+        <f aca="false">Perhitungan!A15</f>
+        <v>10</v>
+      </c>
+      <c r="B16" s="30" t="n">
+        <f aca="false">Perhitungan!M15</f>
+        <v>0.0106992622779771</v>
+      </c>
+      <c r="C16" s="30" t="n">
+        <f aca="false">Perhitungan!E15</f>
+        <v>0.0106382978723404</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
+        <f aca="false">Perhitungan!A16</f>
+        <v>11</v>
+      </c>
+      <c r="B17" s="30" t="n">
+        <f aca="false">Perhitungan!M16</f>
+        <v>0.0142795150829522</v>
+      </c>
+      <c r="C17" s="30" t="n">
+        <f aca="false">Perhitungan!E16</f>
+        <v>0.0140252454417952</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
+        <f aca="false">Perhitungan!A17</f>
+        <v>12</v>
+      </c>
+      <c r="B18" s="30" t="n">
+        <f aca="false">Perhitungan!M17</f>
+        <v>0.0429215375227527</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <f aca="false">Perhitungan!E17</f>
+        <v>0.0427350427350427</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
+        <f aca="false">Perhitungan!A18</f>
+        <v>13</v>
+      </c>
+      <c r="B19" s="30" t="n">
+        <f aca="false">Perhitungan!M18</f>
+        <v>0.0787240655725033</v>
+      </c>
+      <c r="C19" s="30" t="n">
+        <f aca="false">Perhitungan!E18</f>
+        <v>0.078740157480315</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="n">
+        <f aca="false">Perhitungan!A19</f>
+        <v>14</v>
+      </c>
+      <c r="B20" s="30" t="n">
+        <f aca="false">Perhitungan!M19</f>
+        <v>0.114526593622254</v>
+      </c>
+      <c r="C20" s="30" t="n">
+        <f aca="false">Perhitungan!E19</f>
+        <v>0.114503816793893</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="n">
+        <f aca="false">Perhitungan!A20</f>
+        <v>15</v>
+      </c>
+      <c r="B21" s="30" t="n">
+        <f aca="false">Perhitungan!M20</f>
+        <v>0.150329121672005</v>
+      </c>
+      <c r="C21" s="30" t="n">
+        <f aca="false">Perhitungan!E20</f>
+        <v>0.150375939849624</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="n">
+        <f aca="false">Perhitungan!A21</f>
+        <v>16</v>
+      </c>
+      <c r="B22" s="30" t="n">
+        <f aca="false">Perhitungan!M21</f>
+        <v>0.0232763467971916</v>
+      </c>
+      <c r="C22" s="30" t="n">
+        <f aca="false">Perhitungan!E21</f>
+        <v>0.0239234449760766</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="14" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="14" t="n">
+        <f aca="false">1.05*MAX(B7:C22)</f>
+        <v>0.157894736842105</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <f aca="false">B26</f>
+        <v>0.157894736842105</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="n">
+        <f aca="false">Perhitungan!G15</f>
+        <v>0.5</v>
+      </c>
+      <c r="B31" s="30" t="n">
+        <f aca="false">Perhitungan!E15</f>
+        <v>0.0106382978723404</v>
+      </c>
+      <c r="C31" s="30" t="n">
+        <f aca="false">Perhitungan!M15</f>
+        <v>0.0106992622779771</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="n">
+        <f aca="false">Perhitungan!G16</f>
+        <v>1</v>
+      </c>
+      <c r="B32" s="30" t="n">
+        <f aca="false">Perhitungan!E16</f>
+        <v>0.0140252454417952</v>
+      </c>
+      <c r="C32" s="30" t="n">
+        <f aca="false">Perhitungan!M16</f>
+        <v>0.0142795150829522</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="n">
+        <f aca="false">Perhitungan!G17</f>
+        <v>5</v>
+      </c>
+      <c r="B33" s="30" t="n">
+        <f aca="false">Perhitungan!E17</f>
+        <v>0.0427350427350427</v>
+      </c>
+      <c r="C33" s="30" t="n">
+        <f aca="false">Perhitungan!M17</f>
+        <v>0.0429215375227527</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="n">
+        <f aca="false">Perhitungan!G18</f>
+        <v>10</v>
+      </c>
+      <c r="B34" s="30" t="n">
+        <f aca="false">Perhitungan!E18</f>
+        <v>0.078740157480315</v>
+      </c>
+      <c r="C34" s="30" t="n">
+        <f aca="false">Perhitungan!M18</f>
+        <v>0.0787240655725033</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="n">
+        <f aca="false">Perhitungan!G19</f>
+        <v>15</v>
+      </c>
+      <c r="B35" s="30" t="n">
+        <f aca="false">Perhitungan!E19</f>
+        <v>0.114503816793893</v>
+      </c>
+      <c r="C35" s="30" t="n">
+        <f aca="false">Perhitungan!M19</f>
+        <v>0.114526593622254</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10" t="n">
+        <f aca="false">Perhitungan!G20</f>
+        <v>20</v>
+      </c>
+      <c r="B36" s="30" t="n">
+        <f aca="false">Perhitungan!E20</f>
+        <v>0.150375939849624</v>
+      </c>
+      <c r="C36" s="30" t="n">
+        <f aca="false">Perhitungan!M20</f>
+        <v>0.150329121672005</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="29" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="10" t="n">
+        <f aca="false">Perhitungan!F12</f>
+        <v>0</v>
+      </c>
+      <c r="B41" s="30" t="n">
+        <f aca="false">Perhitungan!E12</f>
+        <v>0.0139275766016713</v>
+      </c>
+      <c r="C41" s="30" t="n">
+        <f aca="false">Perhitungan!M12</f>
+        <v>0.0142795150829522</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10" t="n">
+        <f aca="false">Perhitungan!F8</f>
+        <v>1</v>
+      </c>
+      <c r="B42" s="30" t="n">
+        <f aca="false">Perhitungan!E8</f>
+        <v>0.0240384615384615</v>
+      </c>
+      <c r="C42" s="30" t="n">
+        <f aca="false">Perhitungan!M8</f>
+        <v>0.0232763467971916</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="n">
+        <f aca="false">Perhitungan!F9</f>
+        <v>4</v>
+      </c>
+      <c r="B43" s="30" t="n">
+        <f aca="false">Perhitungan!E9</f>
+        <v>0.050761421319797</v>
+      </c>
+      <c r="C43" s="30" t="n">
+        <f aca="false">Perhitungan!M9</f>
+        <v>0.0502668419399101</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="10" t="n">
+        <f aca="false">Perhitungan!F11</f>
+        <v>5</v>
+      </c>
+      <c r="B44" s="30" t="n">
+        <f aca="false">Perhitungan!E11</f>
+        <v>0.0584795321637427</v>
+      </c>
+      <c r="C44" s="30" t="n">
+        <f aca="false">Perhitungan!M11</f>
+        <v>0.0592636736541496</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Compute regression coefficients with corrected-sum formulas b1 = (BC-ED)/(AB-E^2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AkzdwyHYSZDLsThLPh4WDM
</commit_message>
<xml_diff>
--- a/Tabel_10-6_Reaktor_Diferensial.xlsx
+++ b/Tabel_10-6_Reaktor_Diferensial.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="89">
   <si>
     <t xml:space="preserve">Tabel 10-6. Data dari Reaktor Diferensial (Hidrodemetilasi Toluena)</t>
   </si>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">x2²</t>
   </si>
   <si>
-    <t xml:space="preserve">ŷ = a0 + a1·x1 + a2·x2</t>
+    <t xml:space="preserve">ŷ = b0 + b1·x1 + b2·x2</t>
   </si>
   <si>
     <t xml:space="preserve">Residual
@@ -165,49 +165,103 @@
     <t xml:space="preserve">n =</t>
   </si>
   <si>
-    <t xml:space="preserve">Persamaan normal (Cramer):  [A]·[a0; a1; a2] = [b]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matriks A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vektor b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A0 (kolom 1 diganti b)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A1 (kolom 2 diganti b)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A2 (kolom 3 diganti b)</t>
+    <t xml:space="preserve">Jumlah kuadrat terkoreksi (deviasi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A = Σx1²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A = Σx1² − (Σx1)²/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B = Σx2²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B = Σx2² − (Σx2)²/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C = Σx1y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C = Σx1y − (Σx1)(Σy)/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D = Σx2y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D = Σx2y − (Σx2)(Σy)/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E = Σx1x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E = Σx1x2 − (Σx1)(Σx2)/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x̄1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x̄1 = Σx1/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x̄2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x̄2 = Σx2/n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ȳ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ȳ = Σy/n</t>
   </si>
   <si>
     <t xml:space="preserve">Hasil</t>
   </si>
   <si>
-    <t xml:space="preserve">det A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a0 = 1/k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a1 = KB/k</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a2 = KT/k</t>
+    <t xml:space="preserve">AB − E²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">penyebut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b0 = a0 = 1/k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b0 = ȳ − b1·x̄1 − b2·x̄2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b1 = a1 = KB/k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b1 = (BC − ED)/(AB − E²)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b2 = a2 = KT/k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b2 = (AD − EC)/(AB − E²)</t>
   </si>
   <si>
     <t xml:space="preserve">k (× 10^10)</t>
   </si>
   <si>
+    <t xml:space="preserve">k = 1/b0</t>
+  </si>
+  <si>
     <t xml:space="preserve">k (g mol/g kat·s·atm²)</t>
   </si>
   <si>
     <t xml:space="preserve">KB (atm⁻¹)</t>
   </si>
   <si>
+    <t xml:space="preserve">KB = b1/b0</t>
+  </si>
+  <si>
     <t xml:space="preserve">KT (atm⁻¹)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KT = b2/b0</t>
   </si>
   <si>
     <t xml:space="preserve">SSE = Σ(y − ŷ)²</t>
@@ -264,7 +318,7 @@
     <numFmt numFmtId="174" formatCode="0.000"/>
     <numFmt numFmtId="175" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -363,14 +417,22 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <i val="true"/>
       <sz val="9"/>
+      <color rgb="FF555555"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -445,7 +507,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -522,7 +584,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -530,7 +592,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -570,6 +632,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,7 +663,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF878787"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF888888"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
       <rgbColor rgb="FFDDE4EE"/>
@@ -627,7 +693,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF888888"/>
+      <rgbColor rgb="FF555555"/>
       <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -777,11 +843,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1326939"/>
-        <c:axId val="25140594"/>
+        <c:axId val="68254914"/>
+        <c:axId val="92188672"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1326939"/>
+        <c:axId val="68254914"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -848,12 +914,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25140594"/>
+        <c:crossAx val="92188672"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="25140594"/>
+        <c:axId val="92188672"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -930,7 +996,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1326939"/>
+        <c:crossAx val="68254914"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1181,11 +1247,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="11637463"/>
-        <c:axId val="47213593"/>
+        <c:axId val="2351233"/>
+        <c:axId val="94379796"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="11637463"/>
+        <c:axId val="2351233"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1252,12 +1318,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47213593"/>
+        <c:crossAx val="94379796"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47213593"/>
+        <c:axId val="94379796"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1334,7 +1400,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11637463"/>
+        <c:crossAx val="2351233"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1527,11 +1593,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="82038874"/>
-        <c:axId val="50306150"/>
+        <c:axId val="16995849"/>
+        <c:axId val="62727631"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="82038874"/>
+        <c:axId val="16995849"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1598,12 +1664,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50306150"/>
+        <c:crossAx val="62727631"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="50306150"/>
+        <c:axId val="62727631"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1680,7 +1746,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82038874"/>
+        <c:crossAx val="16995849"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1867,11 +1933,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="80747851"/>
-        <c:axId val="81129484"/>
+        <c:axId val="35793490"/>
+        <c:axId val="4514891"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="80747851"/>
+        <c:axId val="35793490"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1938,12 +2004,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81129484"/>
+        <c:crossAx val="4514891"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81129484"/>
+        <c:axId val="4514891"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2020,7 +2086,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80747851"/>
+        <c:crossAx val="35793490"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2350,11 +2416,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="12120149"/>
-        <c:axId val="68585837"/>
+        <c:axId val="15675069"/>
+        <c:axId val="71107463"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="12120149"/>
+        <c:axId val="15675069"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2421,12 +2487,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68585837"/>
+        <c:crossAx val="71107463"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="68585837"/>
+        <c:axId val="71107463"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2503,7 +2569,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12120149"/>
+        <c:crossAx val="15675069"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2820,11 +2886,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="30879269"/>
-        <c:axId val="95176001"/>
+        <c:axId val="37100484"/>
+        <c:axId val="86949441"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="30879269"/>
+        <c:axId val="37100484"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2891,12 +2957,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95176001"/>
+        <c:crossAx val="86949441"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="95176001"/>
+        <c:axId val="86949441"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2973,7 +3039,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30879269"/>
+        <c:crossAx val="37100484"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3266,11 +3332,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="9329568"/>
-        <c:axId val="33116245"/>
+        <c:axId val="98938287"/>
+        <c:axId val="82280152"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="9329568"/>
+        <c:axId val="98938287"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3337,12 +3403,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33116245"/>
+        <c:crossAx val="82280152"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="33116245"/>
+        <c:axId val="82280152"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3419,7 +3485,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9329568"/>
+        <c:crossAx val="98938287"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4629,7 +4695,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -4754,12 +4820,12 @@
         <v>1</v>
       </c>
       <c r="M6" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F6+$C$40*G6</f>
+        <f aca="false">$C$37+$C$38*F6+$C$39*G6</f>
         <v>0.0142795150829522</v>
       </c>
       <c r="N6" s="16" t="n">
         <f aca="false">E6-M6</f>
-        <v>-0.000195008040698632</v>
+        <v>-0.000195008040698634</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4812,12 +4878,12 @@
         <v>1</v>
       </c>
       <c r="M7" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F7+$C$40*G7</f>
+        <f aca="false">$C$37+$C$38*F7+$C$39*G7</f>
         <v>0.0142795150829522</v>
       </c>
       <c r="N7" s="16" t="n">
         <f aca="false">E7-M7</f>
-        <v>-0.000254269641156921</v>
+        <v>-0.000254269641156922</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4870,12 +4936,12 @@
         <v>1</v>
       </c>
       <c r="M8" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F8+$C$40*G8</f>
+        <f aca="false">$C$37+$C$38*F8+$C$39*G8</f>
         <v>0.0232763467971916</v>
       </c>
       <c r="N8" s="16" t="n">
         <f aca="false">E8-M8</f>
-        <v>0.000762114741269901</v>
+        <v>0.000762114741269894</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4928,12 +4994,12 @@
         <v>1</v>
       </c>
       <c r="M9" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F9+$C$40*G9</f>
+        <f aca="false">$C$37+$C$38*F9+$C$39*G9</f>
         <v>0.0502668419399101</v>
       </c>
       <c r="N9" s="16" t="n">
         <f aca="false">E9-M9</f>
-        <v>0.000494579379886874</v>
+        <v>0.000494579379886853</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4986,12 +5052,12 @@
         <v>1</v>
       </c>
       <c r="M10" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F10+$C$40*G10</f>
+        <f aca="false">$C$37+$C$38*F10+$C$39*G10</f>
         <v>0.0232763467971916</v>
       </c>
       <c r="N10" s="16" t="n">
         <f aca="false">E10-M10</f>
-        <v>0.000533177012332173</v>
+        <v>0.000533177012332166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5044,12 +5110,12 @@
         <v>1</v>
       </c>
       <c r="M11" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F11+$C$40*G11</f>
+        <f aca="false">$C$37+$C$38*F11+$C$39*G11</f>
         <v>0.0592636736541496</v>
       </c>
       <c r="N11" s="16" t="n">
         <f aca="false">E11-M11</f>
-        <v>-0.000784141490406877</v>
+        <v>-0.000784141490406898</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5102,12 +5168,12 @@
         <v>1</v>
       </c>
       <c r="M12" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F12+$C$40*G12</f>
+        <f aca="false">$C$37+$C$38*F12+$C$39*G12</f>
         <v>0.0142795150829522</v>
       </c>
       <c r="N12" s="16" t="n">
         <f aca="false">E12-M12</f>
-        <v>-0.000351938481280843</v>
+        <v>-0.000351938481280845</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5160,12 +5226,12 @@
         <v>1</v>
       </c>
       <c r="M13" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F13+$C$40*G13</f>
+        <f aca="false">$C$37+$C$38*F13+$C$39*G13</f>
         <v>0.0142795150829522</v>
       </c>
       <c r="N13" s="16" t="n">
         <f aca="false">E13-M13</f>
-        <v>-0.000195008040698632</v>
+        <v>-0.000195008040698634</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5218,12 +5284,12 @@
         <v>1</v>
       </c>
       <c r="M14" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F14+$C$40*G14</f>
+        <f aca="false">$C$37+$C$38*F14+$C$39*G14</f>
         <v>0.0142795150829522</v>
       </c>
       <c r="N14" s="16" t="n">
         <f aca="false">E14-M14</f>
-        <v>-0.000195008040698632</v>
+        <v>-0.000195008040698634</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5276,12 +5342,12 @@
         <v>0.25</v>
       </c>
       <c r="M15" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F15+$C$40*G15</f>
+        <f aca="false">$C$37+$C$38*F15+$C$39*G15</f>
         <v>0.0106992622779771</v>
       </c>
       <c r="N15" s="16" t="n">
         <f aca="false">E15-M15</f>
-        <v>-6.09644056366616E-005</v>
+        <v>-6.0964405636665E-005</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5334,12 +5400,12 @@
         <v>1</v>
       </c>
       <c r="M16" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F16+$C$40*G16</f>
+        <f aca="false">$C$37+$C$38*F16+$C$39*G16</f>
         <v>0.0142795150829522</v>
       </c>
       <c r="N16" s="16" t="n">
         <f aca="false">E16-M16</f>
-        <v>-0.000254269641156921</v>
+        <v>-0.000254269641156922</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5392,12 +5458,12 @@
         <v>25</v>
       </c>
       <c r="M17" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F17+$C$40*G17</f>
+        <f aca="false">$C$37+$C$38*F17+$C$39*G17</f>
         <v>0.0429215375227527</v>
       </c>
       <c r="N17" s="16" t="n">
         <f aca="false">E17-M17</f>
-        <v>-0.000186494787709941</v>
+        <v>-0.000186494787709948</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5450,7 +5516,7 @@
         <v>100</v>
       </c>
       <c r="M18" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F18+$C$40*G18</f>
+        <f aca="false">$C$37+$C$38*F18+$C$39*G18</f>
         <v>0.0787240655725033</v>
       </c>
       <c r="N18" s="16" t="n">
@@ -5508,12 +5574,12 @@
         <v>225</v>
       </c>
       <c r="M19" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F19+$C$40*G19</f>
+        <f aca="false">$C$37+$C$38*F19+$C$39*G19</f>
         <v>0.114526593622254</v>
       </c>
       <c r="N19" s="16" t="n">
         <f aca="false">E19-M19</f>
-        <v>-2.27768283608681E-005</v>
+        <v>-2.27768283608543E-005</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5566,12 +5632,12 @@
         <v>400</v>
       </c>
       <c r="M20" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F20+$C$40*G20</f>
+        <f aca="false">$C$37+$C$38*F20+$C$39*G20</f>
         <v>0.150329121672005</v>
       </c>
       <c r="N20" s="16" t="n">
         <f aca="false">E20-M20</f>
-        <v>4.68181776194232E-005</v>
+        <v>4.68181776193954E-005</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5624,12 +5690,12 @@
         <v>1</v>
       </c>
       <c r="M21" s="16" t="n">
-        <f aca="false">$C$38+$C$39*F21+$C$40*G21</f>
+        <f aca="false">$C$37+$C$38*F21+$C$39*G21</f>
         <v>0.0232763467971916</v>
       </c>
       <c r="N21" s="16" t="n">
         <f aca="false">E21-M21</f>
-        <v>0.00064709817888492</v>
+        <v>0.000647098178884913</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5682,308 +5748,239 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="19" t="s">
+      <c r="A26" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="F26" s="19" t="s">
+      <c r="C26" s="20" t="n">
+        <f aca="false">$K$22-$F$22^2/$C$22</f>
+        <v>35</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="20" t="n">
-        <f aca="false">$C$22</f>
-        <v>16</v>
+      <c r="A27" s="19" t="s">
+        <v>47</v>
       </c>
       <c r="C27" s="20" t="n">
-        <f aca="false">$F$22</f>
-        <v>12</v>
-      </c>
-      <c r="D27" s="20" t="n">
-        <f aca="false">$G$22</f>
-        <v>61.5</v>
-      </c>
-      <c r="F27" s="20" t="n">
-        <f aca="false">$E$22</f>
-        <v>0.662237227150839</v>
+        <f aca="false">$L$22-$G$22^2/$C$22</f>
+        <v>524.859375</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="20" t="n">
-        <f aca="false">$F$22</f>
-        <v>12</v>
+      <c r="A28" s="19" t="s">
+        <v>49</v>
       </c>
       <c r="C28" s="20" t="n">
-        <f aca="false">$K$22</f>
-        <v>44</v>
-      </c>
-      <c r="D28" s="20" t="n">
-        <f aca="false">$J$22</f>
-        <v>12</v>
-      </c>
-      <c r="F28" s="20" t="n">
-        <f aca="false">$H$22</f>
-        <v>0.567214776421963</v>
+        <f aca="false">$H$22-$F$22*$E$22/$C$22</f>
+        <v>0.0705368560588338</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="20" t="n">
-        <f aca="false">$G$22</f>
-        <v>61.5</v>
+      <c r="A29" s="19" t="s">
+        <v>51</v>
       </c>
       <c r="C29" s="20" t="n">
-        <f aca="false">$J$22</f>
-        <v>12</v>
-      </c>
-      <c r="D29" s="20" t="n">
-        <f aca="false">$L$22</f>
-        <v>761.25</v>
-      </c>
-      <c r="F29" s="20" t="n">
-        <f aca="false">$I$22</f>
-        <v>5.99671595873504</v>
+        <f aca="false">$I$22-$G$22*$E$22/$C$22</f>
+        <v>3.451241616874</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="20" t="n">
+        <f aca="false">$J$22-$F$22*$G$22/$C$22</f>
+        <v>-34.125</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="F31" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="J31" s="19" t="s">
-        <v>49</v>
+      <c r="A31" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="16" t="n">
+        <f aca="false">$F$22/$C$22</f>
+        <v>0.75</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="20" t="n">
-        <f aca="false">$E$22</f>
-        <v>0.662237227150839</v>
-      </c>
-      <c r="C32" s="20" t="n">
-        <f aca="false">$F$22</f>
-        <v>12</v>
-      </c>
-      <c r="D32" s="20" t="n">
-        <f aca="false">$G$22</f>
-        <v>61.5</v>
-      </c>
-      <c r="F32" s="20" t="n">
-        <f aca="false">$C$22</f>
-        <v>16</v>
-      </c>
-      <c r="G32" s="20" t="n">
-        <f aca="false">$E$22</f>
-        <v>0.662237227150839</v>
-      </c>
-      <c r="H32" s="20" t="n">
-        <f aca="false">$G$22</f>
-        <v>61.5</v>
-      </c>
-      <c r="J32" s="20" t="n">
-        <f aca="false">$C$22</f>
-        <v>16</v>
-      </c>
-      <c r="K32" s="20" t="n">
-        <f aca="false">$F$22</f>
-        <v>12</v>
-      </c>
-      <c r="L32" s="20" t="n">
-        <f aca="false">$E$22</f>
-        <v>0.662237227150839</v>
+      <c r="A32" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="16" t="n">
+        <f aca="false">$G$22/$C$22</f>
+        <v>3.84375</v>
+      </c>
+      <c r="D32" s="21" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="20" t="n">
-        <f aca="false">$H$22</f>
-        <v>0.567214776421963</v>
-      </c>
-      <c r="C33" s="20" t="n">
-        <f aca="false">$K$22</f>
-        <v>44</v>
-      </c>
-      <c r="D33" s="20" t="n">
-        <f aca="false">$J$22</f>
-        <v>12</v>
-      </c>
-      <c r="F33" s="20" t="n">
-        <f aca="false">$F$22</f>
-        <v>12</v>
-      </c>
-      <c r="G33" s="20" t="n">
-        <f aca="false">$H$22</f>
-        <v>0.567214776421963</v>
-      </c>
-      <c r="H33" s="20" t="n">
-        <f aca="false">$J$22</f>
-        <v>12</v>
-      </c>
-      <c r="J33" s="20" t="n">
-        <f aca="false">$F$22</f>
-        <v>12</v>
-      </c>
-      <c r="K33" s="20" t="n">
-        <f aca="false">$K$22</f>
-        <v>44</v>
-      </c>
-      <c r="L33" s="20" t="n">
-        <f aca="false">$H$22</f>
-        <v>0.567214776421963</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="20" t="n">
-        <f aca="false">$I$22</f>
-        <v>5.99671595873504</v>
-      </c>
-      <c r="C34" s="20" t="n">
-        <f aca="false">$J$22</f>
-        <v>12</v>
-      </c>
-      <c r="D34" s="20" t="n">
-        <f aca="false">$L$22</f>
-        <v>761.25</v>
-      </c>
-      <c r="F34" s="20" t="n">
-        <f aca="false">$G$22</f>
-        <v>61.5</v>
-      </c>
-      <c r="G34" s="20" t="n">
-        <f aca="false">$I$22</f>
-        <v>5.99671595873504</v>
-      </c>
-      <c r="H34" s="20" t="n">
-        <f aca="false">$L$22</f>
-        <v>761.25</v>
-      </c>
-      <c r="J34" s="20" t="n">
-        <f aca="false">$G$22</f>
-        <v>61.5</v>
-      </c>
-      <c r="K34" s="20" t="n">
-        <f aca="false">$J$22</f>
-        <v>12</v>
-      </c>
-      <c r="L34" s="20" t="n">
-        <f aca="false">$I$22</f>
-        <v>5.99671595873504</v>
+      <c r="A33" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="16" t="n">
+        <f aca="false">$E$22/$C$22</f>
+        <v>0.0413898266969275</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
-        <v>50</v>
+      <c r="A36" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="20" t="n">
+        <f aca="false">C26*C27-C30^2</f>
+        <v>17205.5625</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C37" s="20" t="n">
-        <f aca="false">MDETERM(B27:D29)</f>
-        <v>275289</v>
+      <c r="A37" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" s="22" t="n">
+        <f aca="false">C33-C38*C31-C39*C32</f>
+        <v>0.00711900947300203</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21" t="s">
-        <v>52</v>
+      <c r="A38" s="19" t="s">
+        <v>66</v>
       </c>
       <c r="C38" s="22" t="n">
-        <f aca="false">MDETERM(B32:D34)/C37</f>
-        <v>0.00711900947300202</v>
+        <f aca="false">(C27*C28-C30*C29)/C36</f>
+        <v>0.00899683171423949</v>
+      </c>
+      <c r="D38" s="21" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21" t="s">
-        <v>53</v>
+      <c r="A39" s="19" t="s">
+        <v>68</v>
       </c>
       <c r="C39" s="22" t="n">
-        <f aca="false">MDETERM(F32:H34)/C37</f>
-        <v>0.00899683171423948</v>
+        <f aca="false">(C26*C29-C30*C28)/C36</f>
+        <v>0.00716050560995013</v>
+      </c>
+      <c r="D39" s="21" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="C40" s="22" t="n">
-        <f aca="false">MDETERM(J32:L34)/C37</f>
-        <v>0.00716050560995013</v>
+      <c r="A40" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="23" t="n">
+        <f aca="false">1/C37</f>
+        <v>140.468980100726</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="C41" s="23" t="n">
-        <f aca="false">1/C38</f>
-        <v>140.468980100726</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="C41" s="24" t="n">
+        <f aca="false">C40*0.0000000001</f>
+        <v>1.40468980100726E-008</v>
+      </c>
+      <c r="D41" s="21"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C42" s="24" t="n">
-        <f aca="false">C41*0.0000000001</f>
-        <v>1.40468980100726E-008</v>
+        <v>73</v>
+      </c>
+      <c r="C42" s="25" t="n">
+        <f aca="false">C38/C37</f>
+        <v>1.26377577503709</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="C43" s="25" t="n">
-        <f aca="false">C39/C38</f>
-        <v>1.26377577503709</v>
+        <f aca="false">C39/C37</f>
+        <v>1.00582892003522</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C44" s="25" t="n">
-        <f aca="false">C40/C38</f>
-        <v>1.00582892003522</v>
+      <c r="A44" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="26" t="n">
+        <f aca="false">SUMSQ(N6:N21)</f>
+        <v>2.55203714144949E-006</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="21" t="s">
-        <v>59</v>
+      <c r="A45" s="19" t="s">
+        <v>78</v>
       </c>
       <c r="C45" s="26" t="n">
-        <f aca="false">SUMSQ(N6:N21)</f>
-        <v>2.5520371414495E-006</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C46" s="26" t="n">
         <f aca="false">DEVSQ(E6:E21)</f>
         <v>0.0253497952196739</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C47" s="27" t="n">
-        <f aca="false">1-C45/C46</f>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="27" t="n">
+        <f aca="false">1-C44/C45</f>
         <v>0.999899327110167</v>
       </c>
     </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C48" s="7" t="str">
+        <f aca="false">"y = "&amp;TEXT($C$37,"0.000000")&amp;" + "&amp;TEXT($C$38,"0.000000")&amp;"·x1 + "&amp;TEXT($C$39,"0.000000")&amp;"·x2"</f>
+        <v>y = 0.007119 + 0.008997·x1 + 0.007161·x2</v>
+      </c>
+    </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="s">
-        <v>62</v>
-      </c>
       <c r="C49" s="7" t="str">
-        <f aca="false">"y = "&amp;TEXT($C$38,"0.000000")&amp;" + "&amp;TEXT($C$39,"0.000000")&amp;"·x1 + "&amp;TEXT($C$40,"0.000000")&amp;"·x2"</f>
-        <v>y = 0.007119 + 0.008997·x1 + 0.007161·x2</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C50" s="7" t="str">
-        <f aca="false">"-r'T = "&amp;TEXT(C42,"0.00E+00")&amp;"·PH2·PT / (1 + "&amp;TEXT(C43,"0.000")&amp;"·PB + "&amp;TEXT(C44,"0.000")&amp;"·PT)"</f>
+        <f aca="false">"-r'T = "&amp;TEXT(C41,"0.00E+00")&amp;"·PH2·PT / (1 + "&amp;TEXT(C42,"0.000")&amp;"·PB + "&amp;TEXT(C43,"0.000")&amp;"·PT)"</f>
         <v>-r'T = 1.40E-08·PH2·PT / (1 + 1.264·PB + 1.006·PT)</v>
       </c>
     </row>
@@ -6012,23 +6009,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="str">
-        <f aca="false">"a0 = "&amp;TEXT(Perhitungan!$C$38,"0.000000")&amp;"   a1 = "&amp;TEXT(Perhitungan!$C$39,"0.000000")&amp;"   a2 = "&amp;TEXT(Perhitungan!$C$40,"0.000000")&amp;"   R² = "&amp;TEXT(Perhitungan!C47,"0.0000")</f>
+        <f aca="false">"a0 = "&amp;TEXT(Perhitungan!$C$37,"0.000000")&amp;"   a1 = "&amp;TEXT(Perhitungan!$C$38,"0.000000")&amp;"   a2 = "&amp;TEXT(Perhitungan!$C$39,"0.000000")&amp;"   R² = "&amp;TEXT(Perhitungan!C46,"0.0000")</f>
         <v>a0 = 0.007119   a1 = 0.008997   a2 = 0.007161   R² = 0.9999</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6036,10 +6033,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6267,8 +6264,8 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
-        <v>68</v>
+      <c r="A24" s="31" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6293,7 +6290,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6301,10 +6298,10 @@
         <v>34</v>
       </c>
       <c r="B30" s="29" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6393,7 +6390,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6401,10 +6398,10 @@
         <v>33</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>